<commit_message>
fixing directories part 2
</commit_message>
<xml_diff>
--- a/model makanan/Data Makanan .xlsx
+++ b/model makanan/Data Makanan .xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="bahasa indonesia" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="ENglish" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="238">
   <si>
     <t>Nama Makanan</t>
   </si>
@@ -416,13 +417,322 @@
   </si>
   <si>
     <t>Semua komponen di piring harus diaduk rata ('digado') terlebih dahulu agar setiap sayuran, lontong, dan tahu terlapis oleh saus kacang sebelum dilahap bersama emping melinjo.</t>
+  </si>
+  <si>
+    <t>Chicken braised in a sweet &amp; savory spice paste, grilled over coals.</t>
+  </si>
+  <si>
+    <t>250 kcalPro: 20g | Carb: 10gFat: 14g | Sod: 450mg</t>
+  </si>
+  <si>
+    <t>Soy</t>
+  </si>
+  <si>
+    <t>Chicken, sweet soy sauce, shallots, garlic, coriander</t>
+  </si>
+  <si>
+    <t>Braise with spices till tender. Grill over charcoal, basting with soy sauce.</t>
+  </si>
+  <si>
+    <t>Caramelization over charcoal reflects Javanese patience for sweet results.</t>
+  </si>
+  <si>
+    <t>Best enjoyed muluk (bare hands) with warm rice, sambal, and raw greens.</t>
+  </si>
+  <si>
+    <t>Whole chicken coated in spicy base genep, steamed or slow-roasted.</t>
+  </si>
+  <si>
+    <t>300 kcalPro: 22g | Carb: 8gFat: 18g | Sod: 550mg</t>
+  </si>
+  <si>
+    <t>Peanuts</t>
+  </si>
+  <si>
+    <t>Chicken, base genep (shallots, ginger, turmeric, shrimp paste, lemongrass)</t>
+  </si>
+  <si>
+    <t>Grind spices, coat and stuff chicken. Wrap in banana leaves; steam/slow-roast.</t>
+  </si>
+  <si>
+    <t>Originally for ceremonies. 'Betutu' refers to ancient slow-burning in rice husks.</t>
+  </si>
+  <si>
+    <t>Eaten communally (megibung). Meat is mixed with rice, satay, veggies, and sambal.</t>
+  </si>
+  <si>
+    <t>Yellow-spiced chicken, crispy outside, juicy inside.</t>
+  </si>
+  <si>
+    <t>260 kcalPro: 18g | Carb: 5gFat: 18g | Sod: 300mg</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Chicken, turmeric, garlic, coriander, galangal</t>
+  </si>
+  <si>
+    <t>Boil in yellow spices. Deep-fry until golden brown.</t>
+  </si>
+  <si>
+    <t>Ungkep technique is ancient Sundanese/Javanese wisdom using spices as natural preservatives.</t>
+  </si>
+  <si>
+    <t>Eaten with fingers. Soft bones chewed if free-range. Dipped in cooked sambal terasi.</t>
+  </si>
+  <si>
+    <t>West Sumatra</t>
+  </si>
+  <si>
+    <t>Minang-style boiled chicken, pale but incredibly savory.</t>
+  </si>
+  <si>
+    <t>200 kcalPro: 20g | Carb: 2gFat: 12g | Sod: 350mg</t>
+  </si>
+  <si>
+    <t>Free-range chicken, coconut water, garlic, lime</t>
+  </si>
+  <si>
+    <t>Boil in coconut water &amp; garlic. Briefly dip (10s) in hot oil before serving.</t>
+  </si>
+  <si>
+    <t>Accidental creation in Bukittinggi. 'Pop' because it became highly 'Popular'.</t>
+  </si>
+  <si>
+    <t>Dipped lightly in mild tomato/chili sauce. Served with thin curry broth over rice.</t>
+  </si>
+  <si>
+    <t>Chewy meatballs in a savory beef bone broth.</t>
+  </si>
+  <si>
+    <t>350 kcalPro: 18g | Carb: 45gFat: 12g | Sod: 900mg</t>
+  </si>
+  <si>
+    <t>Gluten, Soy</t>
+  </si>
+  <si>
+    <t>Ground beef, tapioca, garlic, beef bone broth</t>
+  </si>
+  <si>
+    <t>Blend cold beef with ice, garlic, tapioca. Boil meatballs. Serve in marrow broth.</t>
+  </si>
+  <si>
+    <t>Adapted from Chinese pork meatballs (Bak-So) to Halal beef in the archipelago.</t>
+  </si>
+  <si>
+    <t>Customized at the table with soy sauce, sambal, vinegar. Noodles eaten with meat.</t>
+  </si>
+  <si>
+    <t>Makassar, South Sulawesi</t>
+  </si>
+  <si>
+    <t>Beef and offal soup with thick, roasted peanut-spiced broth.</t>
+  </si>
+  <si>
+    <t>400 kcalPro: 25g | Carb: 10gFat: 25g | Sod: 800mg</t>
+  </si>
+  <si>
+    <t>Beef, offal, crushed roasted peanuts, lemongrass, galangal</t>
+  </si>
+  <si>
+    <t>Boil meat with rice water (tajin). Sauté ground spices, add to the broth.</t>
+  </si>
+  <si>
+    <t>Tajin broth is ancient Bugis-Makassar ingenuity to thicken and remove gamey smells.</t>
+  </si>
+  <si>
+    <t>Eaten with halved ketupat or Burasa (coconut milk rice cakes), not plain rice.</t>
+  </si>
+  <si>
+    <t>Broth soup with shredded meat, glass noodles, and veggies.</t>
+  </si>
+  <si>
+    <t>300 kcalPro: 15g | Carb: 20gFat: 12g | Sod: 700mg</t>
+  </si>
+  <si>
+    <t>Eggs, Soy</t>
+  </si>
+  <si>
+    <t>Meat, broth, turmeric, ginger, alliums, celery, glass noodles</t>
+  </si>
+  <si>
+    <t>Boil chicken for broth. Sauté spices, add to boil. Shred chicken, serve with noodles.</t>
+  </si>
+  <si>
+    <t>Influenced by Chinese Caudo and Indian spices. Now has 70+ local variants.</t>
+  </si>
+  <si>
+    <t>Rice often mixed into the bowl. Garnished with lime, sambal, and crushed emping.</t>
+  </si>
+  <si>
+    <t>East Java</t>
+  </si>
+  <si>
+    <t>Beef soup with pitch-black broth from kluwek nuts.</t>
+  </si>
+  <si>
+    <t>350 kcalPro: 20g | Carb: 15gFat: 20g | Sod: 750mg</t>
+  </si>
+  <si>
+    <t>Beef, kluwek nuts, shallots, garlic, coriander, lemongrass</t>
+  </si>
+  <si>
+    <t>Sauté spices with kluwek. Add beef and broth, cook slowly until pitch black.</t>
+  </si>
+  <si>
+    <t>Recorded in 901 AD Taji Inscription; one of Indonesia's oldest dishes.</t>
+  </si>
+  <si>
+    <t>Served with raw short bean sprouts, halved salted egg, and shrimp crackers.</t>
+  </si>
+  <si>
+    <t>Palembang, South Sumatra</t>
+  </si>
+  <si>
+    <t>Chewy fried fish and sago cakes with sour-spicy-sweet cuko sauce.</t>
+  </si>
+  <si>
+    <t>400 kcalPro: 15g | Carb: 50gFat: 15g | Sod: 800mg</t>
+  </si>
+  <si>
+    <t>Fish, Eggs</t>
+  </si>
+  <si>
+    <t>Mackerel, sago flour. Cuko: palm sugar, tamarind, chili, garlic</t>
+  </si>
+  <si>
+    <t>Knead fish with sago. Shape, boil, then fry. Serve with cuko.</t>
+  </si>
+  <si>
+    <t>Created in 16th century by an elderly Chinese man to preserve abundant fish catches.</t>
+  </si>
+  <si>
+    <t>Locals bite the pempek first, then slurp the cuko directly from a small bowl.</t>
+  </si>
+  <si>
+    <t>Beef cooked slowly in coconut milk and spices until dry and preserved.</t>
+  </si>
+  <si>
+    <t>350 kcalPro: 25g | Carb: 10gFat: 25g | Sod: 600mg</t>
+  </si>
+  <si>
+    <t>Beef, thick coconut milk, chili, galangal, ginger, turmeric</t>
+  </si>
+  <si>
+    <t>Cook beef in coconut milk &amp; spices. Stir slowly for hours until dry and caramelized.</t>
+  </si>
+  <si>
+    <t>Born from Minang migration tradition; preserved for long journeys. Crowned world's best food.</t>
+  </si>
+  <si>
+    <t>Eaten dry with warm rice. Leftover spice crumbs (dedak) are mixed with rice.</t>
+  </si>
+  <si>
+    <t>Diced chicken skewers in thick, sweet, savory peanut sauce.</t>
+  </si>
+  <si>
+    <t>400 kcalPro: 25g | Carb: 20gFat: 20g | Sod: 500mg</t>
+  </si>
+  <si>
+    <t>Peanuts, Soy</t>
+  </si>
+  <si>
+    <t>Chicken, peanut sauce, sweet soy sauce, shallots, lime</t>
+  </si>
+  <si>
+    <t>Skewer and grill half-way. Dip in peanut sauce, grill fully. Serve with sauce.</t>
+  </si>
+  <si>
+    <t>Symbol of Madurese persistence; inspired by Arab Kebabs using local peanuts.</t>
+  </si>
+  <si>
+    <t>Meat pulled off with a fork. Plate wiped clean with crackers or lontong.</t>
+  </si>
+  <si>
+    <t>Beef/tongue skewers in thick, spicy yellow/red sauce.</t>
+  </si>
+  <si>
+    <t>350 kcalPro: 25g | Carb: 25gFat: 15g | Sod: 650mg</t>
+  </si>
+  <si>
+    <t>Beef tongue/meat, rice flour, turmeric, coriander, cumin, chili</t>
+  </si>
+  <si>
+    <t>Boil meat in spicy herbs. Skewer and grill briefly. Thicken broth with rice flour.</t>
+  </si>
+  <si>
+    <t>3 sauce colors (Yellow, Red, Brown) reflect Minangkabau flavor diversity.</t>
+  </si>
+  <si>
+    <t>Eaten on banana leaves with katupek, balado cassava chips, or beef skin crackers.</t>
+  </si>
+  <si>
+    <t>Rice stir-fried in a hot wok with seasonings.</t>
+  </si>
+  <si>
+    <t>500 kcalPro: 15g | Carb: 65gFat: 20g | Sod: 800mg</t>
+  </si>
+  <si>
+    <t>Firm white rice, sweet soy sauce, shallots, garlic, chili, egg</t>
+  </si>
+  <si>
+    <t>Sauté spices, scramble egg. Add rice and soy sauce; mix on high heat (wok hei).</t>
+  </si>
+  <si>
+    <t>Originates from Asian philosophy of repurposing leftover cold rice to avoid waste.</t>
+  </si>
+  <si>
+    <t>Served with cucumber-carrot pickles as a palate cleanser and crackers.</t>
+  </si>
+  <si>
+    <t>Young jackfruit cooked slow &amp; sweet with coconut milk.</t>
+  </si>
+  <si>
+    <t>450 kcalPro: 20g | Carb: 45gFat: 20g | Sod: 900mg</t>
+  </si>
+  <si>
+    <t>Eggs</t>
+  </si>
+  <si>
+    <t>Young jackfruit, coconut milk, palm sugar, teak leaves</t>
+  </si>
+  <si>
+    <t>Boil jackfruit, sugar, milk, teak leaves in clay pot on low heat for 12-24 hours.</t>
+  </si>
+  <si>
+    <t>Created in 16th century for workers clearing forests; cooked in large portions.</t>
+  </si>
+  <si>
+    <t>Served Pincuk style on banana leaves. Sweetness balanced with spicy beef skin stew.</t>
+  </si>
+  <si>
+    <t>Nutrient-dense boiled veggies in thick peanut sauce.</t>
+  </si>
+  <si>
+    <t>400 kcalPro: 18g | Carb: 45gFat: 15g | Sod: 600mg</t>
+  </si>
+  <si>
+    <t>Peanuts, Gluten</t>
+  </si>
+  <si>
+    <t>Boiled veggies, tempeh/tofu, ground peanut sauce, palm sugar</t>
+  </si>
+  <si>
+    <t>Boil veggies. Grind peanuts with shrimp paste, sugar, tamarind. Mix evenly.</t>
+  </si>
+  <si>
+    <t>Concocted by 17th-century soldiers mixing leftover peanuts with wild veggies.</t>
+  </si>
+  <si>
+    <t>Must be mixed evenly (digado) before eating with emping crackers.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -432,17 +742,19 @@
     <font>
       <b/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
+      <name val="Google Sans"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Google Sans"/>
+    </font>
+    <font>
+      <color rgb="FF1F1F1F"/>
+      <name val="Google Sans"/>
     </font>
     <font>
       <color theme="1"/>
       <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <color rgb="FF1F1F1F"/>
-      <name val="&quot;Google Sans Text&quot;"/>
     </font>
   </fonts>
   <fills count="3">
@@ -465,12 +777,15 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -479,7 +794,13 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -490,6 +811,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -699,11 +1024,12 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="15.63"/>
-    <col customWidth="1" min="2" max="2" width="19.0"/>
+    <col customWidth="1" min="1" max="1" width="13.38"/>
+    <col customWidth="1" min="2" max="2" width="15.25"/>
     <col customWidth="1" min="3" max="3" width="31.75"/>
     <col customWidth="1" min="4" max="4" width="29.5"/>
-    <col customWidth="1" min="6" max="6" width="18.25"/>
+    <col customWidth="1" min="5" max="5" width="11.75"/>
+    <col customWidth="1" min="6" max="6" width="10.13"/>
     <col customWidth="1" min="7" max="7" width="29.5"/>
     <col customWidth="1" min="8" max="8" width="26.0"/>
     <col customWidth="1" min="9" max="9" width="26.25"/>
@@ -726,7 +1052,7 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -743,483 +1069,1023 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="2">
+      <c r="F2" s="3">
         <v>2.0</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="3">
         <v>5.0</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="3">
         <v>1.0</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="5" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="3">
         <v>1.0</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="5" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="2">
+      <c r="F6" s="3">
         <v>1.0</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="5" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="3">
         <v>2.0</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="5" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="3">
         <v>1.0</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G8" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="3">
         <v>1.0</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="3">
         <v>4.0</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="G10" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="H10" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="5" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="3">
         <v>4.0</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="5" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="E12" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="F12" s="2">
+      <c r="F12" s="3">
         <v>1.0</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="G12" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="H12" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="5" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="E13" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="F13" s="2">
+      <c r="F13" s="3">
         <v>4.0</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="H13" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="E14" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F14" s="2">
+      <c r="F14" s="3">
         <v>3.0</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="G14" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H14" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="5" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="E15" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="F15" s="2">
+      <c r="F15" s="3">
         <v>1.0</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="G15" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="H15" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E16" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="F16" s="2">
+      <c r="F16" s="3">
         <v>2.0</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="G16" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="H16" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>134</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="1" horizontalCentered="1"/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup fitToHeight="0" cellComments="atEnd" orientation="landscape" pageOrder="overThenDown"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="13.38"/>
+    <col customWidth="1" min="2" max="2" width="15.25"/>
+    <col customWidth="1" min="3" max="3" width="31.75"/>
+    <col customWidth="1" min="4" max="4" width="29.5"/>
+    <col customWidth="1" min="5" max="5" width="11.75"/>
+    <col customWidth="1" min="6" max="6" width="10.13"/>
+    <col customWidth="1" min="7" max="7" width="29.5"/>
+    <col customWidth="1" min="8" max="8" width="26.0"/>
+    <col customWidth="1" min="9" max="9" width="26.25"/>
+    <col customWidth="1" min="10" max="10" width="40.63"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F2" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F3" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F4" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F5" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F7" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F8" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F9" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="F10" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F11" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="F12" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F13" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F14" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="F15" s="7">
+        <v>1.0</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="F16" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>237</v>
       </c>
     </row>
   </sheetData>

</xml_diff>